<commit_message>
Automate sprint ticket FOUR-189
</commit_message>
<xml_diff>
--- a/data/TestExcel (1).xlsx
+++ b/data/TestExcel (1).xlsx
@@ -55,14 +55,13 @@
     <t>Service &amp; Maintenance</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/service-and-maintenance.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/service-&amp;-maintenance.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/service-and-maintainance.svg</t>
   </si>
   <si>
-    <t xml:space="preserve"> 
-Gurugram</t>
+    <t>gurugram</t>
   </si>
   <si>
     <t>Affordable Car Service &amp; Maintenance in Gurugram | Fourdoor</t>
@@ -83,14 +82,25 @@
     <t>AC Service &amp; Repair</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/ac-service-&amp;-repair.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/ac-service--&amp;-repair.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/ac-service-&amp;-repair.svg</t>
   </si>
   <si>
-    <t xml:space="preserve">Best Car AC Service in Gurugram by Fourdoor - Stay Cool and Comfortable
+    <r>
+      <t>Best Car AC Service in Gurugram by Fourdoor - Stay Cool and Comfortable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
 </t>
+    </r>
   </si>
   <si>
     <t>Stay cool with Fourdoor's car AC service in Gurugram. Expert solutions for a comfortable drive every time.</t>
@@ -108,7 +118,7 @@
     <t>General Inspection</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/general-inspection.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/general-inspection.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/general-inspection.svg</t>
@@ -132,7 +142,7 @@
     <t>Denting &amp; Painting</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/body-shop-dent-&amp;-paint.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/body-shop-dent-&amp;-paint.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/body-shop-dent-&amp;-paint.svg</t>
@@ -156,7 +166,7 @@
     <t>Steering &amp; Suspension</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/streeing-&amp;-suspension.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/steering-&amp;-suspension.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/sterring-&amp;-suspension.svg</t>
@@ -180,7 +190,7 @@
     <t>Engine &amp; Brakes</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/engine-&amp;-brakes.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/engine-&amp;-brakes.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/super-category-banner.svg</t>
@@ -204,7 +214,7 @@
     <t>Car Detailing</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/car-detailing.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/car-detailing.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/detailing.svg</t>
@@ -213,8 +223,7 @@
     <t>Professional Car Detailing in Gurugram - Fourdoor Experts</t>
   </si>
   <si>
-    <t xml:space="preserve">Transform your car with Fourdoor's detailing services in Gurugram. Premium service for a pristine look inside and out.
-</t>
+    <t>Transform your car with Fourdoor's detailing services in Gurugram. Premium service for a pristine look inside and out.</t>
   </si>
   <si>
     <t>Transform Your Car with Fourdoor's Detailing Service</t>
@@ -229,7 +238,7 @@
     <t>Car Wash &amp; Spa</t>
   </si>
   <si>
-    <t>https://media.fourdoor.com/fourdoor-images/super-category-icons/car-wash.svg</t>
+    <t>https://media.fourdoor.dev/fourdoor-images/super-category-icons/car-wash-&amp;-spa.png</t>
   </si>
   <si>
     <t>https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/car-wash-&amp;-spa-02.svg</t>
@@ -249,31 +258,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9"/>
-      <color rgb="FF1155CC"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -281,20 +277,149 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="9"/>
-      <color rgb="FF1155CC"/>
-      <name val="Monaco"/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -306,135 +431,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -447,6 +444,13 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -457,8 +461,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FF00FF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -469,19 +521,115 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -499,161 +647,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -674,30 +717,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -708,16 +727,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </left>
       <right style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </right>
       <top style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -741,184 +760,195 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="31" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1184,8 +1214,9 @@
   <dimension ref="A1:V9"/>
   <sheetFormatPr defaultColWidth="12.6339285714286" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="4" max="4" width="42.1339285714286" customWidth="1"/>
-    <col min="5" max="5" width="40.25" customWidth="1"/>
+    <col min="4" max="4" width="78.4196428571429" customWidth="1"/>
+    <col min="5" max="5" width="54.4642857142857" customWidth="1"/>
+    <col min="6" max="6" width="22.4642857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:22">
@@ -1201,22 +1232,22 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1"/>
@@ -1245,22 +1276,22 @@
       <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="8">
         <v>1</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="K2" s="1"/>
@@ -1286,26 +1317,25 @@
       <c r="C3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="10">
-        <f t="shared" ref="G3:G9" si="0">SUM(G2+1)</f>
+      <c r="G3" s="8">
         <v>2</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="1" t="s">
         <v>26</v>
       </c>
       <c r="K3" s="1"/>
@@ -1331,26 +1361,25 @@
       <c r="C4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="10">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="H4" s="6" t="s">
+      <c r="G4" s="8">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="1" t="s">
         <v>34</v>
       </c>
       <c r="K4" s="1"/>
@@ -1376,26 +1405,25 @@
       <c r="C5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="10">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="H5" s="6" t="s">
+      <c r="G5" s="8">
+        <v>3</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="1" t="s">
         <v>42</v>
       </c>
       <c r="K5" s="1"/>
@@ -1421,26 +1449,25 @@
       <c r="C6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="10">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H6" s="6" t="s">
+      <c r="G6" s="8">
+        <v>6</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K6" s="1"/>
@@ -1466,26 +1493,25 @@
       <c r="C7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="10">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="H7" s="6" t="s">
+      <c r="G7" s="8">
+        <v>7</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="1" t="s">
         <v>58</v>
       </c>
       <c r="K7" s="1"/>
@@ -1511,26 +1537,25 @@
       <c r="C8" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="10">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="H8" s="6" t="s">
+      <c r="G8" s="8">
+        <v>4</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="1" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="1"/>
@@ -1556,26 +1581,25 @@
       <c r="C9" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="10">
-        <f t="shared" si="0"/>
+      <c r="G9" s="8">
         <v>8</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="1" t="s">
         <v>74</v>
       </c>
       <c r="K9" s="1"/>
@@ -1593,22 +1617,22 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/service-and-maintenance.svg"/>
-    <hyperlink ref="E2" r:id="rId2" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/service-and-maintainance.svg"/>
-    <hyperlink ref="D3" r:id="rId3" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/ac-service-&amp;-repair.svg"/>
-    <hyperlink ref="E3" r:id="rId4" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/ac-service-&amp;-repair.svg"/>
-    <hyperlink ref="D4" r:id="rId5" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/general-inspection.svg"/>
-    <hyperlink ref="E4" r:id="rId6" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/general-inspection.svg"/>
-    <hyperlink ref="D5" r:id="rId7" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/body-shop-dent-&amp;-paint.svg"/>
-    <hyperlink ref="E5" r:id="rId8" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/body-shop-dent-&amp;-paint.svg"/>
-    <hyperlink ref="D6" r:id="rId9" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/streeing-&amp;-suspension.svg"/>
-    <hyperlink ref="E6" r:id="rId10" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/sterring-&amp;-suspension.svg"/>
-    <hyperlink ref="D7" r:id="rId11" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/engine-&amp;-brakes.svg"/>
-    <hyperlink ref="E7" r:id="rId12" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/super-category-banner.svg"/>
-    <hyperlink ref="D8" r:id="rId13" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/car-detailing.svg"/>
-    <hyperlink ref="E8" r:id="rId14" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/detailing.svg"/>
-    <hyperlink ref="D9" r:id="rId15" display="https://media.fourdoor.com/fourdoor-images/super-category-icons/car-wash.svg"/>
-    <hyperlink ref="E9" r:id="rId16" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/car-wash-&amp;-spa-02.svg"/>
+    <hyperlink ref="D2" r:id="rId1" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/service-&amp;-maintenance.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/service-&amp;-maintenance.png"/>
+    <hyperlink ref="E2" r:id="rId2" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/service-and-maintainance.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/super-category_svg-banner/service-and-maintainance.svg"/>
+    <hyperlink ref="D3" r:id="rId3" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/ac-service--&amp;-repair.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/ac-service--&amp;-repair.png"/>
+    <hyperlink ref="E3" r:id="rId4" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/ac-service-&amp;-repair.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/ac-service-&amp;-repair.jpg"/>
+    <hyperlink ref="D4" r:id="rId5" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/general-inspection.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/general-inspection.png"/>
+    <hyperlink ref="E4" r:id="rId6" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/general-inspection.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/general-inspection.jpg"/>
+    <hyperlink ref="D5" r:id="rId7" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/body-shop-dent-&amp;-paint.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/body-shop-dent-&amp;-paint.png"/>
+    <hyperlink ref="E5" r:id="rId8" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/body-shop-dent-&amp;-paint.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/bodyshop-dent-&amp;-paint.jpg"/>
+    <hyperlink ref="D6" r:id="rId9" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/steering-&amp;-suspension.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/steering-&amp;-suspension.png"/>
+    <hyperlink ref="E6" r:id="rId10" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/sterring-&amp;-suspension.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/steering-&amp;-suspension.jpg"/>
+    <hyperlink ref="D7" r:id="rId11" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/engine-&amp;-brakes.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/engine-&amp;-brakes.png"/>
+    <hyperlink ref="E7" r:id="rId12" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/super-category-banner.svg" tooltip="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/super-category-banner.svg"/>
+    <hyperlink ref="D8" r:id="rId13" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/car-detailing.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/car-detailing.png"/>
+    <hyperlink ref="E8" r:id="rId14" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/detailing.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/detailing.jpg"/>
+    <hyperlink ref="D9" r:id="rId15" display="https://media.fourdoor.dev/fourdoor-images/super-category-icons/car-wash-&amp;-spa.png" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-icons/car-wash-&amp;-spa.png"/>
+    <hyperlink ref="E9" r:id="rId16" display="https://media.fourdoor.com/fourdoor-images/super-category-banners/super-category_svg-banner/car-wash-&amp;-spa-02.svg" tooltip="https://media.fourdoor.dev/fourdoor-images/super-category-banners/car-wash-&amp;-spa.jpg"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>